<commit_message>
Obra de los cuestionarios brutal
</commit_message>
<xml_diff>
--- a/krm/static/files/import_questionnaire.xlsx
+++ b/krm/static/files/import_questionnaire.xlsx
@@ -5,49 +5,54 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bienvenidosaez/Bitbucket/krm-kpmg/krm/static/files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bienvenidosaez/Proyectos/KPMG_KRM/_import/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{454998E9-A0A9-824D-8CB8-A39A481B00AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D880537-0101-1E4D-8A39-D8C17B185E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30720" yWindow="500" windowWidth="40960" windowHeight="23880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51200" yWindow="500" windowWidth="35840" windowHeight="21900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="QUESTIONNAIRES" sheetId="4" r:id="rId1"/>
+    <sheet name="SCOPES" sheetId="3" r:id="rId2"/>
+    <sheet name="QUESTIONS" sheetId="2" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$1</definedName>
-  </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
-    <t>DELEGACION</t>
+    <t>SCOPE_REF</t>
   </si>
   <si>
-    <t>CONCESION</t>
+    <t>SCOPE_NAME</t>
   </si>
   <si>
-    <t>AREA</t>
+    <t>SCOPE_USERS_EMAILS</t>
   </si>
   <si>
-    <t>PREGUNTA</t>
+    <t>QUESTION_REF</t>
   </si>
   <si>
-    <t>USUARIO/EMAIL</t>
+    <t>QUESTION_TITLE</t>
   </si>
   <si>
-    <t>REF</t>
+    <t>SCOPES_REFS</t>
+  </si>
+  <si>
+    <t>QUESTIONNAIRE_REF</t>
+  </si>
+  <si>
+    <t>QUESTIONNAIRE_NAME</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -63,6 +68,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -72,7 +85,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -95,17 +108,54 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="8"/>
+      </left>
+      <right style="thin">
+        <color theme="8"/>
+      </right>
+      <top style="thin">
+        <color theme="8"/>
+      </top>
+      <bottom style="thin">
+        <color theme="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -441,40 +491,824 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D110B751-E793-5A4A-BF8F-1A7C629C83D5}">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.5" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="31.83203125" customWidth="1"/>
-    <col min="4" max="4" width="29.5" customWidth="1"/>
-    <col min="5" max="5" width="149.5" customWidth="1"/>
-    <col min="6" max="6" width="27.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8684F057-C68B-8842-ACAB-BC8EA111E45B}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="64.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D2" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70D15546-EFCA-1641-9F4F-2EA62F7C9B2A}">
+  <dimension ref="A1:C149"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="26.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="12.5" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="83.5" style="7" customWidth="1"/>
+    <col min="3" max="3" width="79.83203125" style="7" customWidth="1"/>
+    <col min="4" max="16384" width="26.33203125" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="6"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="6"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="6"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="6"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="6"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="6"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="6"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="6"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="6"/>
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="6"/>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="6"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="6"/>
+      <c r="B39" s="6"/>
+      <c r="C39" s="6"/>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="6"/>
+      <c r="B40" s="6"/>
+      <c r="C40" s="6"/>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" s="6"/>
+      <c r="B41" s="6"/>
+      <c r="C41" s="6"/>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="6"/>
+      <c r="B42" s="6"/>
+      <c r="C42" s="6"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" s="6"/>
+      <c r="B43" s="6"/>
+      <c r="C43" s="6"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" s="6"/>
+      <c r="B44" s="6"/>
+      <c r="C44" s="6"/>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" s="6"/>
+      <c r="B45" s="6"/>
+      <c r="C45" s="6"/>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" s="6"/>
+      <c r="B46" s="6"/>
+      <c r="C46" s="6"/>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" s="6"/>
+      <c r="B47" s="6"/>
+      <c r="C47" s="6"/>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" s="6"/>
+      <c r="B48" s="6"/>
+      <c r="C48" s="6"/>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" s="6"/>
+      <c r="B49" s="6"/>
+      <c r="C49" s="6"/>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" s="6"/>
+      <c r="B50" s="6"/>
+      <c r="C50" s="6"/>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" s="6"/>
+      <c r="B51" s="6"/>
+      <c r="C51" s="6"/>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" s="6"/>
+      <c r="B52" s="6"/>
+      <c r="C52" s="6"/>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53" s="6"/>
+      <c r="B53" s="6"/>
+      <c r="C53" s="6"/>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" s="6"/>
+      <c r="B54" s="6"/>
+      <c r="C54" s="6"/>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" s="6"/>
+      <c r="B55" s="6"/>
+      <c r="C55" s="6"/>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" s="6"/>
+      <c r="B56" s="6"/>
+      <c r="C56" s="6"/>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" s="6"/>
+      <c r="B57" s="6"/>
+      <c r="C57" s="6"/>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" s="6"/>
+      <c r="B58" s="6"/>
+      <c r="C58" s="6"/>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" s="6"/>
+      <c r="B59" s="6"/>
+      <c r="C59" s="6"/>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="6"/>
+      <c r="B60" s="6"/>
+      <c r="C60" s="6"/>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="6"/>
+      <c r="B61" s="6"/>
+      <c r="C61" s="6"/>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="6"/>
+      <c r="B62" s="6"/>
+      <c r="C62" s="6"/>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="6"/>
+      <c r="B63" s="6"/>
+      <c r="C63" s="6"/>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="6"/>
+      <c r="B64" s="6"/>
+      <c r="C64" s="6"/>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="6"/>
+      <c r="B65" s="6"/>
+      <c r="C65" s="6"/>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="6"/>
+      <c r="B66" s="6"/>
+      <c r="C66" s="6"/>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="6"/>
+      <c r="B67" s="6"/>
+      <c r="C67" s="6"/>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="6"/>
+      <c r="B68" s="6"/>
+      <c r="C68" s="6"/>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="6"/>
+      <c r="B69" s="6"/>
+      <c r="C69" s="6"/>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="6"/>
+      <c r="B70" s="6"/>
+      <c r="C70" s="6"/>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="6"/>
+      <c r="B71" s="6"/>
+      <c r="C71" s="6"/>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" s="6"/>
+      <c r="B72" s="6"/>
+      <c r="C72" s="6"/>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" s="6"/>
+      <c r="B73" s="6"/>
+      <c r="C73" s="6"/>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74" s="6"/>
+      <c r="B74" s="6"/>
+      <c r="C74" s="6"/>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75" s="6"/>
+      <c r="B75" s="6"/>
+      <c r="C75" s="6"/>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76" s="6"/>
+      <c r="B76" s="6"/>
+      <c r="C76" s="6"/>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77" s="6"/>
+      <c r="B77" s="6"/>
+      <c r="C77" s="6"/>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A78" s="6"/>
+      <c r="B78" s="6"/>
+      <c r="C78" s="6"/>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A79" s="6"/>
+      <c r="B79" s="6"/>
+      <c r="C79" s="6"/>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A80" s="6"/>
+      <c r="B80" s="6"/>
+      <c r="C80" s="6"/>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A81" s="6"/>
+      <c r="B81" s="6"/>
+      <c r="C81" s="6"/>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A82" s="6"/>
+      <c r="B82" s="6"/>
+      <c r="C82" s="6"/>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A83" s="6"/>
+      <c r="B83" s="6"/>
+      <c r="C83" s="6"/>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A84" s="6"/>
+      <c r="B84" s="6"/>
+      <c r="C84" s="6"/>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A85" s="6"/>
+      <c r="B85" s="6"/>
+      <c r="C85" s="6"/>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A86" s="6"/>
+      <c r="B86" s="6"/>
+      <c r="C86" s="6"/>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A87" s="6"/>
+      <c r="B87" s="6"/>
+      <c r="C87" s="6"/>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A88" s="6"/>
+      <c r="B88" s="6"/>
+      <c r="C88" s="6"/>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A89" s="6"/>
+      <c r="B89" s="6"/>
+      <c r="C89" s="6"/>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A90" s="6"/>
+      <c r="B90" s="6"/>
+      <c r="C90" s="6"/>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A91" s="6"/>
+      <c r="B91" s="6"/>
+      <c r="C91" s="6"/>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A92" s="6"/>
+      <c r="B92" s="6"/>
+      <c r="C92" s="6"/>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A93" s="6"/>
+      <c r="B93" s="6"/>
+      <c r="C93" s="6"/>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A94" s="6"/>
+      <c r="B94" s="6"/>
+      <c r="C94" s="6"/>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A95" s="6"/>
+      <c r="B95" s="6"/>
+      <c r="C95" s="6"/>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A96" s="6"/>
+      <c r="B96" s="6"/>
+      <c r="C96" s="6"/>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A97" s="6"/>
+      <c r="B97" s="6"/>
+      <c r="C97" s="6"/>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A98" s="6"/>
+      <c r="B98" s="6"/>
+      <c r="C98" s="6"/>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A99" s="6"/>
+      <c r="B99" s="6"/>
+      <c r="C99" s="6"/>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A100" s="6"/>
+      <c r="B100" s="6"/>
+      <c r="C100" s="6"/>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A101" s="6"/>
+      <c r="B101" s="6"/>
+      <c r="C101" s="6"/>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A102" s="6"/>
+      <c r="B102" s="6"/>
+      <c r="C102" s="6"/>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A103" s="6"/>
+      <c r="B103" s="6"/>
+      <c r="C103" s="6"/>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A104" s="6"/>
+      <c r="B104" s="6"/>
+      <c r="C104" s="6"/>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A105" s="6"/>
+      <c r="B105" s="6"/>
+      <c r="C105" s="6"/>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A106" s="6"/>
+      <c r="B106" s="6"/>
+      <c r="C106" s="6"/>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A107" s="6"/>
+      <c r="B107" s="6"/>
+      <c r="C107" s="6"/>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A108" s="6"/>
+      <c r="B108" s="6"/>
+      <c r="C108" s="6"/>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A109" s="6"/>
+      <c r="B109" s="6"/>
+      <c r="C109" s="6"/>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A110" s="6"/>
+      <c r="B110" s="6"/>
+      <c r="C110" s="6"/>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A111" s="6"/>
+      <c r="B111" s="6"/>
+      <c r="C111" s="6"/>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A112" s="6"/>
+      <c r="B112" s="6"/>
+      <c r="C112" s="6"/>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A113" s="6"/>
+      <c r="B113" s="6"/>
+      <c r="C113" s="6"/>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A114" s="6"/>
+      <c r="B114" s="6"/>
+      <c r="C114" s="6"/>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A115" s="6"/>
+      <c r="B115" s="6"/>
+      <c r="C115" s="6"/>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A116" s="6"/>
+      <c r="B116" s="6"/>
+      <c r="C116" s="6"/>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A117" s="6"/>
+      <c r="B117" s="6"/>
+      <c r="C117" s="6"/>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A118" s="6"/>
+      <c r="B118" s="6"/>
+      <c r="C118" s="6"/>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A119" s="6"/>
+      <c r="B119" s="6"/>
+      <c r="C119" s="6"/>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A120" s="6"/>
+      <c r="B120" s="6"/>
+      <c r="C120" s="6"/>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A121" s="6"/>
+      <c r="B121" s="6"/>
+      <c r="C121" s="6"/>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A122" s="6"/>
+      <c r="B122" s="6"/>
+      <c r="C122" s="6"/>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A123" s="6"/>
+      <c r="B123" s="6"/>
+      <c r="C123" s="6"/>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A124" s="6"/>
+      <c r="B124" s="6"/>
+      <c r="C124" s="6"/>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A125" s="6"/>
+      <c r="B125" s="6"/>
+      <c r="C125" s="6"/>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A126" s="6"/>
+      <c r="B126" s="6"/>
+      <c r="C126" s="6"/>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A127" s="6"/>
+      <c r="B127" s="6"/>
+      <c r="C127" s="6"/>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A128" s="6"/>
+      <c r="B128" s="6"/>
+      <c r="C128" s="6"/>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A129" s="6"/>
+      <c r="B129" s="6"/>
+      <c r="C129" s="6"/>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A130" s="6"/>
+      <c r="B130" s="6"/>
+      <c r="C130" s="6"/>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A131" s="6"/>
+      <c r="B131" s="6"/>
+      <c r="C131" s="6"/>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A132" s="6"/>
+      <c r="B132" s="6"/>
+      <c r="C132" s="6"/>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A133" s="6"/>
+      <c r="B133" s="6"/>
+      <c r="C133" s="6"/>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A134" s="6"/>
+      <c r="B134" s="6"/>
+      <c r="C134" s="6"/>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A135" s="6"/>
+      <c r="B135" s="6"/>
+      <c r="C135" s="6"/>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A136" s="6"/>
+      <c r="B136" s="6"/>
+      <c r="C136" s="6"/>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A137" s="6"/>
+      <c r="B137" s="6"/>
+      <c r="C137" s="6"/>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A138" s="6"/>
+      <c r="B138" s="6"/>
+      <c r="C138" s="6"/>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A139" s="6"/>
+      <c r="B139" s="6"/>
+      <c r="C139" s="6"/>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A140" s="6"/>
+      <c r="B140" s="6"/>
+      <c r="C140" s="6"/>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A141" s="6"/>
+      <c r="B141" s="6"/>
+      <c r="C141" s="6"/>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A142" s="6"/>
+      <c r="B142" s="6"/>
+      <c r="C142" s="6"/>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A143" s="6"/>
+      <c r="B143" s="6"/>
+      <c r="C143" s="6"/>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A144" s="6"/>
+      <c r="B144" s="6"/>
+      <c r="C144" s="6"/>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A145" s="6"/>
+      <c r="B145" s="6"/>
+      <c r="C145" s="6"/>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A146" s="6"/>
+      <c r="B146" s="6"/>
+      <c r="C146" s="6"/>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A147" s="6"/>
+      <c r="B147" s="6"/>
+      <c r="C147" s="6"/>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A148" s="6"/>
+      <c r="B148" s="6"/>
+      <c r="C148" s="6"/>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A149" s="6"/>
+      <c r="B149" s="6"/>
+      <c r="C149" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>